<commit_message>
Added DateEntry widget which is not working as expected in updating the underlying variable when a new date is selected
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results__COPY.xlsx
+++ b/rss_islandr/templates/results__COPY.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="0" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="41">
   <si>
     <t>Soil</t>
   </si>
@@ -137,22 +137,16 @@
     <t>Industrial</t>
   </si>
   <si>
-    <t>Industrial waste</t>
-  </si>
-  <si>
-    <t>Small</t>
+    <t>Toxic metals</t>
   </si>
   <si>
     <t>Medium</t>
   </si>
   <si>
+    <t>No limit to access</t>
+  </si>
+  <si>
     <t>High</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>No limit to access</t>
   </si>
   <si>
     <t>&lt;1m</t>
@@ -687,7 +681,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -780,6 +774,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Calculation" xfId="3" builtinId="22"/>
@@ -1138,7 +1133,9 @@
       <c r="B3" s="33"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
+      <c r="E3" s="44">
+        <v>42038</v>
+      </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -1236,7 +1233,7 @@
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1257,7 +1254,7 @@
       </c>
       <c r="B9" s="35"/>
       <c r="C9" s="5">
-        <v>0.27999999999999903</v>
+        <v>0.48999999999999899</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -1324,7 +1321,7 @@
       </c>
       <c r="B12" s="31"/>
       <c r="C12" s="18" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D12" s="30" t="s">
         <v>9</v>
@@ -1361,7 +1358,7 @@
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="18" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D13" s="32" t="s">
         <v>15</v>
@@ -1398,7 +1395,7 @@
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="18" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D14" s="32" t="s">
         <v>19</v>
@@ -1472,7 +1469,7 @@
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="18" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D16" s="34" t="s">
         <v>10</v>
@@ -1505,7 +1502,7 @@
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="10">
-        <v>1</v>
+        <v>0.48999999999999899</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
@@ -1651,7 +1648,7 @@
       </c>
       <c r="B22" s="43"/>
       <c r="C22" s="19">
-        <v>0.13999999999999899</v>
+        <v>0</v>
       </c>
       <c r="D22" s="42" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Implementation of read/write scenario
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results__COPY.xlsx
+++ b/rss_islandr/templates/results__COPY.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="36">
   <si>
     <t>Soil</t>
   </si>
@@ -135,21 +135,6 @@
   </si>
   <si>
     <t>Industrial</t>
-  </si>
-  <si>
-    <t>Toxic metals</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>No limit to access</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>&lt;1m</t>
   </si>
 </sst>
 </file>
@@ -1191,7 +1176,7 @@
       </c>
       <c r="B6" s="37"/>
       <c r="C6" s="18" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1212,7 +1197,7 @@
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1233,7 +1218,7 @@
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1254,7 +1239,7 @@
       </c>
       <c r="B9" s="35"/>
       <c r="C9" s="5">
-        <v>0.48999999999999899</v>
+        <v>0</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -1321,7 +1306,7 @@
       </c>
       <c r="B12" s="31"/>
       <c r="C12" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D12" s="30" t="s">
         <v>9</v>
@@ -1358,7 +1343,7 @@
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D13" s="32" t="s">
         <v>15</v>
@@ -1395,7 +1380,7 @@
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="18" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D14" s="32" t="s">
         <v>19</v>
@@ -1432,7 +1417,7 @@
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D15" s="32" t="s">
         <v>20</v>
@@ -1469,7 +1454,7 @@
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="18" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="D16" s="34" t="s">
         <v>10</v>
@@ -1502,7 +1487,7 @@
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="10">
-        <v>0.48999999999999899</v>
+        <v>0</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>

</xml_diff>

<commit_message>
The source-pathways and partially the receptor meters are automatically updated through the use of traces
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results__COPY.xlsx
+++ b/rss_islandr/templates/results__COPY.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="50">
   <si>
     <t>Soil</t>
   </si>
@@ -125,9 +125,6 @@
     <t>Total Risk</t>
   </si>
   <si>
-    <t>Value Not Known</t>
-  </si>
-  <si>
     <t>Significant waterway</t>
   </si>
   <si>
@@ -135,6 +132,51 @@
   </si>
   <si>
     <t>Industrial</t>
+  </si>
+  <si>
+    <t>Bio-accumulative and toxic materials</t>
+  </si>
+  <si>
+    <t>Large</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>No limit to access</t>
+  </si>
+  <si>
+    <t>&lt;1m</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>5m</t>
+  </si>
+  <si>
+    <t>Silt/clay aquifer: 20m</t>
+  </si>
+  <si>
+    <t>Area source</t>
+  </si>
+  <si>
+    <t>&lt;1km</t>
+  </si>
+  <si>
+    <t>PM10</t>
+  </si>
+  <si>
+    <t>Frequent</t>
+  </si>
+  <si>
+    <t>Gravel</t>
+  </si>
+  <si>
+    <t>Domestic/potable</t>
   </si>
 </sst>
 </file>
@@ -1176,7 +1218,7 @@
       </c>
       <c r="B6" s="37"/>
       <c r="C6" s="18" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1197,7 +1239,7 @@
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="18" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1218,7 +1260,7 @@
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="18" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1239,7 +1281,7 @@
       </c>
       <c r="B9" s="35"/>
       <c r="C9" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -1306,35 +1348,35 @@
       </c>
       <c r="B12" s="31"/>
       <c r="C12" s="18" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="31"/>
       <c r="F12" s="18" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="G12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="H12" s="31"/>
       <c r="I12" s="16" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="J12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="K12" s="31"/>
       <c r="L12" s="16" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="M12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="N12" s="31"/>
       <c r="O12" s="16" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1343,35 +1385,35 @@
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="18" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D13" s="32" t="s">
         <v>15</v>
       </c>
       <c r="E13" s="33"/>
       <c r="F13" s="18" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="G13" s="32" t="s">
         <v>15</v>
       </c>
       <c r="H13" s="33"/>
       <c r="I13" s="17" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="J13" s="36" t="s">
         <v>22</v>
       </c>
       <c r="K13" s="37"/>
       <c r="L13" s="17" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="M13" s="36" t="s">
         <v>25</v>
       </c>
       <c r="N13" s="37"/>
       <c r="O13" s="17" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -1380,35 +1422,35 @@
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D14" s="32" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="33"/>
       <c r="F14" s="18" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="G14" s="32" t="s">
         <v>21</v>
       </c>
       <c r="H14" s="33"/>
       <c r="I14" s="17" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="J14" s="36" t="s">
         <v>23</v>
       </c>
       <c r="K14" s="37"/>
       <c r="L14" s="17" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="M14" s="36" t="s">
         <v>26</v>
       </c>
       <c r="N14" s="37"/>
       <c r="O14" s="17" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1417,35 +1459,35 @@
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="18" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D15" s="32" t="s">
         <v>20</v>
       </c>
       <c r="E15" s="33"/>
       <c r="F15" s="18" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="G15" s="34" t="s">
         <v>10</v>
       </c>
       <c r="H15" s="35"/>
       <c r="I15" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" s="36" t="s">
         <v>24</v>
       </c>
       <c r="K15" s="37"/>
       <c r="L15" s="17" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="M15" s="36" t="s">
         <v>27</v>
       </c>
       <c r="N15" s="37"/>
       <c r="O15" s="17" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1454,14 +1496,14 @@
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="18" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D16" s="34" t="s">
         <v>10</v>
       </c>
       <c r="E16" s="35"/>
       <c r="F16" s="11">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="1"/>
@@ -1471,14 +1513,14 @@
       </c>
       <c r="K16" s="35"/>
       <c r="L16" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M16" s="34" t="s">
         <v>10</v>
       </c>
       <c r="N16" s="35"/>
       <c r="O16" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1487,7 +1529,7 @@
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="10">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
@@ -1580,14 +1622,14 @@
       </c>
       <c r="K20" s="41"/>
       <c r="L20" s="18" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" s="40" t="s">
         <v>29</v>
       </c>
       <c r="N20" s="41"/>
       <c r="O20" s="17" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -1596,35 +1638,35 @@
       </c>
       <c r="B21" s="33"/>
       <c r="C21" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="E21" s="33"/>
       <c r="F21" s="18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="H21" s="33"/>
       <c r="I21" s="18" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="J21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="K21" s="33"/>
       <c r="L21" s="18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="N21" s="33"/>
       <c r="O21" s="17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1633,35 +1675,35 @@
       </c>
       <c r="B22" s="43"/>
       <c r="C22" s="19">
-        <v>0</v>
+        <v>0.35</v>
       </c>
       <c r="D22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="E22" s="43"/>
       <c r="F22" s="19">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="G22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="H22" s="43"/>
       <c r="I22" s="19">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="J22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="K22" s="43"/>
       <c r="L22" s="19">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="M22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="N22" s="43"/>
       <c r="O22" s="10">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Minor additions. Version increased (previous commit)
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results__COPY.xlsx
+++ b/rss_islandr/templates/results__COPY.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="36">
   <si>
     <t>Soil</t>
   </si>
@@ -125,6 +125,9 @@
     <t>Total Risk</t>
   </si>
   <si>
+    <t>Value Not Known</t>
+  </si>
+  <si>
     <t>Significant waterway</t>
   </si>
   <si>
@@ -132,51 +135,6 @@
   </si>
   <si>
     <t>Industrial</t>
-  </si>
-  <si>
-    <t>Bio-accumulative and toxic materials</t>
-  </si>
-  <si>
-    <t>Large</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>No limit to access</t>
-  </si>
-  <si>
-    <t>&lt;1m</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>5m</t>
-  </si>
-  <si>
-    <t>Silt/clay aquifer: 20m</t>
-  </si>
-  <si>
-    <t>Area source</t>
-  </si>
-  <si>
-    <t>&lt;1km</t>
-  </si>
-  <si>
-    <t>PM10</t>
-  </si>
-  <si>
-    <t>Frequent</t>
-  </si>
-  <si>
-    <t>Gravel</t>
-  </si>
-  <si>
-    <t>Domestic/potable</t>
   </si>
 </sst>
 </file>
@@ -1161,7 +1119,7 @@
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="44">
-        <v>42038</v>
+        <v>45834</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
@@ -1218,7 +1176,7 @@
       </c>
       <c r="B6" s="37"/>
       <c r="C6" s="18" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1239,7 +1197,7 @@
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="18" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1260,7 +1218,7 @@
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1281,7 +1239,7 @@
       </c>
       <c r="B9" s="35"/>
       <c r="C9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -1348,35 +1306,35 @@
       </c>
       <c r="B12" s="31"/>
       <c r="C12" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="31"/>
       <c r="F12" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="H12" s="31"/>
       <c r="I12" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="J12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="K12" s="31"/>
       <c r="L12" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="M12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="N12" s="31"/>
       <c r="O12" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1385,35 +1343,35 @@
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="18" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D13" s="32" t="s">
         <v>15</v>
       </c>
       <c r="E13" s="33"/>
       <c r="F13" s="18" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="G13" s="32" t="s">
         <v>15</v>
       </c>
       <c r="H13" s="33"/>
       <c r="I13" s="17" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="J13" s="36" t="s">
         <v>22</v>
       </c>
       <c r="K13" s="37"/>
       <c r="L13" s="17" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="M13" s="36" t="s">
         <v>25</v>
       </c>
       <c r="N13" s="37"/>
       <c r="O13" s="17" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -1422,35 +1380,35 @@
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="18" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D14" s="32" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="33"/>
       <c r="F14" s="18" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="G14" s="32" t="s">
         <v>21</v>
       </c>
       <c r="H14" s="33"/>
       <c r="I14" s="17" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="J14" s="36" t="s">
         <v>23</v>
       </c>
       <c r="K14" s="37"/>
       <c r="L14" s="17" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="M14" s="36" t="s">
         <v>26</v>
       </c>
       <c r="N14" s="37"/>
       <c r="O14" s="17" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1459,35 +1417,35 @@
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="18" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D15" s="32" t="s">
         <v>20</v>
       </c>
       <c r="E15" s="33"/>
       <c r="F15" s="18" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="G15" s="34" t="s">
         <v>10</v>
       </c>
       <c r="H15" s="35"/>
       <c r="I15" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" s="36" t="s">
         <v>24</v>
       </c>
       <c r="K15" s="37"/>
       <c r="L15" s="17" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="M15" s="36" t="s">
         <v>27</v>
       </c>
       <c r="N15" s="37"/>
       <c r="O15" s="17" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1496,14 +1454,14 @@
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="18" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="D16" s="34" t="s">
         <v>10</v>
       </c>
       <c r="E16" s="35"/>
       <c r="F16" s="11">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="1"/>
@@ -1513,14 +1471,14 @@
       </c>
       <c r="K16" s="35"/>
       <c r="L16" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M16" s="34" t="s">
         <v>10</v>
       </c>
       <c r="N16" s="35"/>
       <c r="O16" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1529,7 +1487,7 @@
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="10">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
@@ -1622,14 +1580,14 @@
       </c>
       <c r="K20" s="41"/>
       <c r="L20" s="18" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M20" s="40" t="s">
         <v>29</v>
       </c>
       <c r="N20" s="41"/>
       <c r="O20" s="17" t="s">
-        <v>14</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -1638,35 +1596,35 @@
       </c>
       <c r="B21" s="33"/>
       <c r="C21" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="E21" s="33"/>
       <c r="F21" s="18" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="H21" s="33"/>
       <c r="I21" s="18" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="J21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="K21" s="33"/>
       <c r="L21" s="18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="N21" s="33"/>
       <c r="O21" s="17" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1675,35 +1633,35 @@
       </c>
       <c r="B22" s="43"/>
       <c r="C22" s="19">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="D22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="E22" s="43"/>
       <c r="F22" s="19">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="H22" s="43"/>
       <c r="I22" s="19">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="J22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="K22" s="43"/>
       <c r="L22" s="19">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="M22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="N22" s="43"/>
       <c r="O22" s="10">
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Selection of skin color improved significanlty
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results__COPY.xlsx
+++ b/rss_islandr/templates/results__COPY.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="0" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -666,7 +666,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -759,7 +759,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Calculation" xfId="3" builtinId="22"/>
@@ -1118,9 +1117,7 @@
       <c r="B3" s="33"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
-      <c r="E3" s="44">
-        <v>45834</v>
-      </c>
+      <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>

</xml_diff>

<commit_message>
Added a mechanism to read lat, (long) from map
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results__COPY.xlsx
+++ b/rss_islandr/templates/results__COPY.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="44">
   <si>
     <t>Soil</t>
   </si>
@@ -135,6 +135,30 @@
   </si>
   <si>
     <t>Industrial</t>
+  </si>
+  <si>
+    <t>Industrial waste</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>No limit to access</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>&lt;1m</t>
   </si>
 </sst>
 </file>
@@ -1120,7 +1144,9 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="H3" s="1">
+        <v>38.272689999999997</v>
+      </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -1173,7 +1199,7 @@
       </c>
       <c r="B6" s="37"/>
       <c r="C6" s="18" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1194,7 +1220,7 @@
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="18" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1215,7 +1241,7 @@
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="18" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1236,7 +1262,7 @@
       </c>
       <c r="B9" s="35"/>
       <c r="C9" s="5">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -1303,7 +1329,7 @@
       </c>
       <c r="B12" s="31"/>
       <c r="C12" s="18" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D12" s="30" t="s">
         <v>9</v>
@@ -1340,7 +1366,7 @@
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="18" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D13" s="32" t="s">
         <v>15</v>
@@ -1377,7 +1403,7 @@
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="18" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="D14" s="32" t="s">
         <v>19</v>
@@ -1414,7 +1440,7 @@
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="18" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="D15" s="32" t="s">
         <v>20</v>
@@ -1451,7 +1477,7 @@
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="18" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="D16" s="34" t="s">
         <v>10</v>
@@ -1484,7 +1510,7 @@
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="10">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
@@ -1630,28 +1656,28 @@
       </c>
       <c r="B22" s="43"/>
       <c r="C22" s="19">
-        <v>0</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="D22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="E22" s="43"/>
       <c r="F22" s="19">
-        <v>0</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="G22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="H22" s="43"/>
       <c r="I22" s="19">
-        <v>0</v>
+        <v>9.6000000000000002E-2</v>
       </c>
       <c r="J22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="K22" s="43"/>
       <c r="L22" s="19">
-        <v>0</v>
+        <v>2.8799999999999999E-2</v>
       </c>
       <c r="M22" s="42" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
BUG FIX: map.html was not fetching coordinates because webview was not being made ready immediately
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/results__COPY.xlsx
+++ b/rss_islandr/templates/results__COPY.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="49">
   <si>
     <t>Soil</t>
   </si>
@@ -125,30 +125,12 @@
     <t>Total Risk</t>
   </si>
   <si>
-    <t>Value Not Known</t>
-  </si>
-  <si>
     <t>Significant waterway</t>
   </si>
   <si>
     <t>Option 1</t>
   </si>
   <si>
-    <t>Industrial</t>
-  </si>
-  <si>
-    <t>this is it</t>
-  </si>
-  <si>
-    <t>Analysts</t>
-  </si>
-  <si>
-    <t>Agricultural areas - Arable Land</t>
-  </si>
-  <si>
-    <t>CLAY - sandy clay</t>
-  </si>
-  <si>
     <t>Bio-accumulative and toxic materials</t>
   </si>
   <si>
@@ -158,13 +140,40 @@
     <t>High</t>
   </si>
   <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>No limit to access</t>
+  </si>
+  <si>
+    <t>&lt;1m</t>
+  </si>
+  <si>
+    <t>Unconfined</t>
+  </si>
+  <si>
+    <t>Silt/clay aquifer: 20m</t>
+  </si>
+  <si>
     <t>Medium</t>
   </si>
   <si>
-    <t>No limit to access</t>
-  </si>
-  <si>
-    <t>&lt;1m</t>
+    <t>Point source</t>
+  </si>
+  <si>
+    <t>&lt;1km</t>
+  </si>
+  <si>
+    <t>PM10</t>
+  </si>
+  <si>
+    <t>Frequent</t>
+  </si>
+  <si>
+    <t>Gravel</t>
+  </si>
+  <si>
+    <t>Commercial</t>
   </si>
 </sst>
 </file>
@@ -696,7 +705,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -789,7 +798,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Calculation" xfId="3" builtinId="22"/>
@@ -1127,18 +1135,14 @@
         <v>3</v>
       </c>
       <c r="B2" s="37"/>
-      <c r="C2" s="2" t="s">
-        <v>36</v>
-      </c>
+      <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="2" t="s">
-        <v>38</v>
-      </c>
+      <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
@@ -1152,18 +1156,14 @@
       <c r="B3" s="33"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
-      <c r="E3" s="44">
-        <v>45771</v>
-      </c>
+      <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1">
-        <v>58.85</v>
+        <v>0</v>
       </c>
       <c r="I3" s="1"/>
-      <c r="J3" s="1" t="s">
-        <v>39</v>
-      </c>
+      <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
@@ -1175,15 +1175,13 @@
         <v>5</v>
       </c>
       <c r="B4" s="39"/>
-      <c r="C4" s="4" t="s">
-        <v>37</v>
-      </c>
+      <c r="C4" s="4"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4">
-        <v>45.69</v>
+        <v>0</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
@@ -1218,7 +1216,7 @@
       </c>
       <c r="B6" s="37"/>
       <c r="C6" s="18" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1239,7 +1237,7 @@
       </c>
       <c r="B7" s="33"/>
       <c r="C7" s="18" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1260,7 +1258,7 @@
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="18" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1348,35 +1346,35 @@
       </c>
       <c r="B12" s="31"/>
       <c r="C12" s="18" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="31"/>
       <c r="F12" s="18" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="H12" s="31"/>
       <c r="I12" s="16" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="K12" s="31"/>
       <c r="L12" s="16" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="M12" s="30" t="s">
         <v>9</v>
       </c>
       <c r="N12" s="31"/>
       <c r="O12" s="16" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1385,35 +1383,35 @@
       </c>
       <c r="B13" s="33"/>
       <c r="C13" s="18" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D13" s="32" t="s">
         <v>15</v>
       </c>
       <c r="E13" s="33"/>
       <c r="F13" s="18" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="G13" s="32" t="s">
         <v>15</v>
       </c>
       <c r="H13" s="33"/>
       <c r="I13" s="17" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="J13" s="36" t="s">
         <v>22</v>
       </c>
       <c r="K13" s="37"/>
       <c r="L13" s="17" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="M13" s="36" t="s">
         <v>25</v>
       </c>
       <c r="N13" s="37"/>
       <c r="O13" s="17" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -1422,35 +1420,35 @@
       </c>
       <c r="B14" s="33"/>
       <c r="C14" s="18" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D14" s="32" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="33"/>
       <c r="F14" s="18" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="G14" s="32" t="s">
         <v>21</v>
       </c>
       <c r="H14" s="33"/>
       <c r="I14" s="17" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J14" s="36" t="s">
         <v>23</v>
       </c>
       <c r="K14" s="37"/>
       <c r="L14" s="17" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="M14" s="36" t="s">
         <v>26</v>
       </c>
       <c r="N14" s="37"/>
       <c r="O14" s="17" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1459,35 +1457,35 @@
       </c>
       <c r="B15" s="33"/>
       <c r="C15" s="18" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D15" s="32" t="s">
         <v>20</v>
       </c>
       <c r="E15" s="33"/>
       <c r="F15" s="18" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="G15" s="34" t="s">
         <v>10</v>
       </c>
       <c r="H15" s="35"/>
       <c r="I15" s="11">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="J15" s="36" t="s">
         <v>24</v>
       </c>
       <c r="K15" s="37"/>
       <c r="L15" s="17" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="M15" s="36" t="s">
         <v>27</v>
       </c>
       <c r="N15" s="37"/>
       <c r="O15" s="17" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1496,14 +1494,14 @@
       </c>
       <c r="B16" s="21"/>
       <c r="C16" s="18" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D16" s="34" t="s">
         <v>10</v>
       </c>
       <c r="E16" s="35"/>
       <c r="F16" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="15"/>
       <c r="H16" s="1"/>
@@ -1513,14 +1511,14 @@
       </c>
       <c r="K16" s="35"/>
       <c r="L16" s="11">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="M16" s="34" t="s">
         <v>10</v>
       </c>
       <c r="N16" s="35"/>
       <c r="O16" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1529,7 +1527,7 @@
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="10">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="13"/>
@@ -1601,7 +1599,7 @@
       </c>
       <c r="B20" s="41"/>
       <c r="C20" s="18" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D20" s="40" t="s">
         <v>29</v>
@@ -1638,35 +1636,35 @@
       </c>
       <c r="B21" s="33"/>
       <c r="C21" s="18" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="D21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="E21" s="33"/>
       <c r="F21" s="18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="H21" s="33"/>
       <c r="I21" s="18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="K21" s="33"/>
       <c r="L21" s="18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M21" s="32" t="s">
         <v>30</v>
       </c>
       <c r="N21" s="33"/>
       <c r="O21" s="17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1675,35 +1673,35 @@
       </c>
       <c r="B22" s="43"/>
       <c r="C22" s="19">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="D22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="E22" s="43"/>
       <c r="F22" s="19">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="G22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="H22" s="43"/>
       <c r="I22" s="19">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="J22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="K22" s="43"/>
       <c r="L22" s="19">
-        <v>0.21</v>
+        <v>0.3</v>
       </c>
       <c r="M22" s="42" t="s">
         <v>31</v>
       </c>
       <c r="N22" s="43"/>
       <c r="O22" s="10">
-        <v>0</v>
+        <v>0.21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>